<commit_message>
Simplify worker import template
</commit_message>
<xml_diff>
--- a/templates/Mau_nhap_danh_sach_cong_nhan.xlsx
+++ b/templates/Mau_nhap_danh_sach_cong_nhan.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh sach CBCNV" sheetId="1" r:id="R0646188ea21f4ae9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh sach CBCNV" sheetId="1" r:id="Rbc5436066b5149d6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -239,58 +239,58 @@
   <x:sheetData>
     <x:row r="1" ht="19.5" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>Họ tên</x:v>
+        <x:v>Số thứ tự</x:v>
       </x:c>
       <x:c r="B1" s="4" t="str">
-        <x:v>Năm sinh</x:v>
-      </x:c>
-      <x:c r="C1" s="6" t="str">
+        <x:v>Họ và tên</x:v>
+      </x:c>
+      <x:c r="C1" s="4" t="str">
+        <x:v>Bộ phận</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
         <x:v>Số điện thoại</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
-        <x:v>Bộ phận</x:v>
-      </x:c>
     </x:row>
     <x:row r="2" ht="19.5" customHeight="1">
-      <x:c r="A2" s="5" t="str">
+      <x:c r="A2" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" s="5" t="str">
         <x:v>Nguyễn Văn A</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="str">
-        <x:v>1990</x:v>
-      </x:c>
       <x:c r="C2" s="5" t="str">
+        <x:v>May 1</x:v>
+      </x:c>
+      <x:c r="D2" s="5" t="str">
         <x:v>0901000001</x:v>
       </x:c>
-      <x:c r="D2" s="5" t="str">
-        <x:v>May 1</x:v>
-      </x:c>
     </x:row>
     <x:row r="3" ht="19.5" customHeight="1">
-      <x:c r="A3" s="5" t="str">
+      <x:c r="A3" s="5" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="5" t="str">
         <x:v>Trần Thị B</x:v>
       </x:c>
-      <x:c r="B3" s="5" t="str">
-        <x:v>1992</x:v>
-      </x:c>
       <x:c r="C3" s="5" t="str">
+        <x:v>May 2</x:v>
+      </x:c>
+      <x:c r="D3" s="5" t="str">
         <x:v>0901000002</x:v>
       </x:c>
-      <x:c r="D3" s="5" t="str">
-        <x:v>May 2</x:v>
-      </x:c>
     </x:row>
     <x:row r="4" ht="19.5" customHeight="1">
-      <x:c r="A4" s="5" t="str">
+      <x:c r="A4" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="5" t="str">
         <x:v>Lê Văn C</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="str">
-        <x:v>1988</x:v>
-      </x:c>
       <x:c r="C4" s="5" t="str">
+        <x:v>Cơ điện</x:v>
+      </x:c>
+      <x:c r="D4" s="5" t="str">
         <x:v>0901000003</x:v>
-      </x:c>
-      <x:c r="D4" s="5" t="str">
-        <x:v>Cơ điện</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>